<commit_message>
Schedule posts for 23-25 Oct; update plan and posts list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014eEsgB524rBa4fvKpZHVjX
</commit_message>
<xml_diff>
--- a/plan/content_plan.xlsx
+++ b/plan/content_plan.xlsx
@@ -1115,7 +1115,7 @@
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Scheduled 23 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1213,7 @@
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Scheduled 24 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1262,7 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Scheduled 25 Oct 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Schedule one-hand fold (28 Oct) and next car seat (29 Oct) posts; update plan and posts list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012esCAN3xr8hWB3UX9QHEof
</commit_message>
<xml_diff>
--- a/plan/content_plan.xlsx
+++ b/plan/content_plan.xlsx
@@ -1406,10 +1406,14 @@
           <t>Pram folded</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>https://babysorted.com/article?slug=stroller-test-checklist</t>
+        </is>
+      </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Scheduled 28 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -1455,10 +1459,14 @@
           <t>Toddler car seat</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>https://babysorted.com/article?slug=car-seat-groups-guide</t>
+        </is>
+      </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Scheduled 29 Oct 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Schedule nursery mistakes (30 Oct), baby bottles (31 Oct), Bugaboo Fox vs Butterfly (1 Nov); update plan and posts list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012esCAMPbkxNus5E6wvwUHy
</commit_message>
<xml_diff>
--- a/plan/content_plan.xlsx
+++ b/plan/content_plan.xlsx
@@ -1512,10 +1512,14 @@
           <t>Nursery set</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>https://babysorted.com/article?slug=safe-sleep-setup-checklist</t>
+        </is>
+      </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Scheduled 30 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -1659,10 +1663,14 @@
           <t>Bottles</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>https://babysorted.com/article?slug=baby-bottle-buying-guide</t>
+        </is>
+      </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Scheduled 31 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -1708,10 +1716,14 @@
           <t>Both models</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>https://babysorted.com/article?slug=travel-stroller-buying-guide</t>
+        </is>
+      </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Scheduled 1 Nov 2026</t>
         </is>
       </c>
     </row>

</xml_diff>